<commit_message>
Add AI Insights composite scoring, KB recommendations, SLA/escalation, comms monitoring, manager risk view, and suggested workflows
Builds out the FEI Insights backlog: renamed/reframed the AI note (AI Insights,
probable-cause framing), composite confidence scoring across routing/diagnosis/
recommendation/similarity, engineer track record + shift-aware handoff risk,
insight cards, historical routing consistency, a new KB article catalog with
similarity+success-rate ranking and per-article feedback (with next-best
suggestion on dislike), SLA tiers/timers with escalation reminders, a
communication-gap monitor with progress-aware templates, a manager risk view,
and a clearly-labeled (non-executed) suggested-workflow section.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/engineer_roster.xlsx
+++ b/backend/data/engineer_roster.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,16 @@
           <t>On-call</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Resolved Count</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Avg Resolution (hrs)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -543,6 +553,12 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N2" t="n">
+        <v>52</v>
+      </c>
+      <c r="O2" t="n">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -604,6 +620,12 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N3" t="n">
+        <v>28</v>
+      </c>
+      <c r="O3" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -665,6 +687,12 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N4" t="n">
+        <v>31</v>
+      </c>
+      <c r="O4" t="n">
+        <v>6.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -726,6 +754,12 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N5" t="n">
+        <v>47</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -787,6 +821,12 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N6" t="n">
+        <v>24</v>
+      </c>
+      <c r="O6" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -848,6 +888,12 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N7" t="n">
+        <v>26</v>
+      </c>
+      <c r="O7" t="n">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -909,6 +955,12 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N8" t="n">
+        <v>55</v>
+      </c>
+      <c r="O8" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -970,6 +1022,12 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N9" t="n">
+        <v>22</v>
+      </c>
+      <c r="O9" t="n">
+        <v>8.5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1031,6 +1089,12 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N10" t="n">
+        <v>9</v>
+      </c>
+      <c r="O10" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1092,6 +1156,12 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N11" t="n">
+        <v>49</v>
+      </c>
+      <c r="O11" t="n">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1153,6 +1223,12 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N12" t="n">
+        <v>25</v>
+      </c>
+      <c r="O12" t="n">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1214,6 +1290,12 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N13" t="n">
+        <v>11</v>
+      </c>
+      <c r="O13" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1275,6 +1357,12 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N14" t="n">
+        <v>27</v>
+      </c>
+      <c r="O14" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1336,6 +1424,12 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N15" t="n">
+        <v>23</v>
+      </c>
+      <c r="O15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1396,6 +1490,12 @@
         <is>
           <t>No</t>
         </is>
+      </c>
+      <c r="N16" t="n">
+        <v>10</v>
+      </c>
+      <c r="O16" t="n">
+        <v>11.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Phase 1 — Dynamics 365 Finance domain expansion
- roster.py: added 6 Finance team aliases (GL, AP, AR, Fixed Assets,
  Inventory/Warehouse, Batch Jobs/Integration) to _TEAM_ALIASES so
  Finance tickets route to the right engineers automatically
- orchestrator.py: made missing-info detection domain-aware — Finance
  tickets now check for legal entity, Finance module, infolog error,
  and voucher number instead of Kubernetes fields; added _detect_domain()
  to classify tickets by keyword matching
- seed_kb_articles.py: added 6 Finance KB articles covering vendor invoice
  posting, GL journal unbalanced voucher, fixed asset depreciation, customer
  payment settlement, DMF import staging error, and inventory negative quantity
- engineer_roster.xlsx: added 8 Finance engineers (3×L1, 3×L2, 2×L3) across
  AP, AR, GL, Inventory, and Batch Jobs/Integration specialties

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/engineer_roster.xlsx
+++ b/backend/data/engineer_roster.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1498,6 +1498,494 @@
         <v>11.5</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Priya Sharma</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>priya.sharma@questsupport.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>09:00-18:00</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Accounts Payable</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>ap,vendor,invoice,payment,voucher</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>18</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ravi Nair</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ravi.nair@questsupport.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>09:00-18:00</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Accounts Receivable</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>ar,customer invoice,collection,aging,dunning</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>5</v>
+      </c>
+      <c r="L18" t="n">
+        <v>3</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>21</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Meera Pillai</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>meera.pillai@questsupport.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Asia/Colombo</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>08:00-17:00</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Inventory / Warehouse</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>inventory,warehouse,wms,stock,bom,item</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>5</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>15</v>
+      </c>
+      <c r="O19" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Anand Krishnan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>anand.krishnan@questsupport.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>10:00-19:00</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>General Ledger / Accounting</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>gl,ledger,journal,posting,fiscal,accounting,coa</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>6</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>44</v>
+      </c>
+      <c r="O20" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Divya Menon</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>divya.menon@questsupport.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Europe/London</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>08:00-17:00</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Accounts Payable</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>ap,vendor,invoice,payment,voucher,po,three-way match</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>6</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>39</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Karthik Rajan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>karthik.rajan@questsupport.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Asia/Singapore</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>09:00-18:00</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Batch Jobs / Integration</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>batch,integration,dmf,data entity,odata,import,export</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>6</v>
+      </c>
+      <c r="L22" t="n">
+        <v>4</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>31</v>
+      </c>
+      <c r="O22" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Suresh Babu</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>suresh.babu@questsupport.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>09:00-18:00</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>General Ledger / Accounting</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>gl,ledger,journal,fiscal,period close,coa,fixed asset,depreciation</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>4</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>87</v>
+      </c>
+      <c r="O23" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lakshmi Narayanan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>lakshmi.n@questsupport.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Europe/Amsterdam</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>08:00-17:00</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Batch Jobs / Integration</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>batch,integration,dmf,data entity,odata,d365 finance,erp</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>4</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>72</v>
+      </c>
+      <c r="O24" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>